<commit_message>
imported round 19 bets
</commit_message>
<xml_diff>
--- a/uploads/sportsbet.xlsx
+++ b/uploads/sportsbet.xlsx
@@ -15,7 +15,7 @@
     <sheet state="visible" name="Playoffs" sheetId="10" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Transaction History'!$A$1:$U$194</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Transaction History'!$A$1:$U$202</definedName>
   </definedNames>
   <calcPr/>
   <pivotCaches>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="182">
   <si>
     <t>Time (AEST)</t>
   </si>
@@ -541,6 +541,34 @@
   </si>
   <si>
     <t>Carlton v Hawthorn
+ Same Game Multi</t>
+  </si>
+  <si>
+    <t>Sydney Swans v Adelaide Crows
+ Same Game Multi</t>
+  </si>
+  <si>
+    <t>Geelong Cats v St Kilda
+ Same Game Multi</t>
+  </si>
+  <si>
+    <t>Collingwood v Carlton
+ Same Game Multi</t>
+  </si>
+  <si>
+    <t>North Melbourne v Melbourne
+ Same Game Multi</t>
+  </si>
+  <si>
+    <t>Gold Coast SUNS v Western Bulldogs
+ Same Game Multi</t>
+  </si>
+  <si>
+    <t>West Coast Eagles v Brisbane Lions
+ Same Game Multi</t>
+  </si>
+  <si>
+    <t>Essendon v GWS GIANTS
  Same Game Multi</t>
   </si>
   <si>
@@ -1161,11 +1189,11 @@
           </c:val>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="196508934"/>
-        <c:axId val="1639401484"/>
+        <c:axId val="167968187"/>
+        <c:axId val="1734051455"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="196508934"/>
+        <c:axId val="167968187"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1221,10 +1249,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1639401484"/>
+        <c:crossAx val="1734051455"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1639401484"/>
+        <c:axId val="1734051455"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1301,7 +1329,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="196508934"/>
+        <c:crossAx val="167968187"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1442,11 +1470,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="932573680"/>
-        <c:axId val="1837428422"/>
+        <c:axId val="373592461"/>
+        <c:axId val="1867424185"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="932573680"/>
+        <c:axId val="373592461"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1502,10 +1530,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1837428422"/>
+        <c:crossAx val="1867424185"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1837428422"/>
+        <c:axId val="1867424185"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1517,7 +1545,7 @@
             <a:noFill/>
           </a:ln>
         </c:spPr>
-        <c:crossAx val="932573680"/>
+        <c:crossAx val="373592461"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -9608,28 +9636,308 @@
       </c>
     </row>
     <row r="195" ht="15.75" customHeight="1">
-      <c r="A195" s="1"/>
+      <c r="A195" s="4">
+        <v>46217.51111111111</v>
+      </c>
+      <c r="B195" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C195" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D195" s="8">
+        <v>9.459159638E9</v>
+      </c>
+      <c r="E195" s="8">
+        <v>6.945105761E9</v>
+      </c>
+      <c r="F195" s="8">
+        <v>-33.0</v>
+      </c>
+      <c r="G195" s="8">
+        <v>291.7</v>
+      </c>
+      <c r="H195" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I195" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J195" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K195" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L195" s="10" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="196" ht="15.75" customHeight="1">
-      <c r="A196" s="1"/>
+      <c r="A196" s="4">
+        <v>46218.89166666667</v>
+      </c>
+      <c r="B196" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C196" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D196" s="8">
+        <v>9.462931717E9</v>
+      </c>
+      <c r="E196" s="8">
+        <v>6.947833679E9</v>
+      </c>
+      <c r="F196" s="8">
+        <v>-33.0</v>
+      </c>
+      <c r="G196" s="8">
+        <v>258.7</v>
+      </c>
+      <c r="H196" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I196" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J196" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K196" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L196" s="10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="197" ht="15.75" customHeight="1">
-      <c r="A197" s="1"/>
+      <c r="A197" s="4">
+        <v>46219.9375</v>
+      </c>
+      <c r="B197" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C197" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="D197" s="8">
+        <v>9.466391174E9</v>
+      </c>
+      <c r="E197" s="8">
+        <v>6.950280154E9</v>
+      </c>
+      <c r="F197" s="8">
+        <v>-32.0</v>
+      </c>
+      <c r="G197" s="8">
+        <v>226.7</v>
+      </c>
+      <c r="H197" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I197" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J197" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K197" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L197" s="10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="198" ht="15.75" customHeight="1">
-      <c r="A198" s="1"/>
+      <c r="A198" s="4">
+        <v>46220.95208333333</v>
+      </c>
+      <c r="B198" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C198" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D198" s="8">
+        <v>9.469762331E9</v>
+      </c>
+      <c r="E198" s="8">
+        <v>6.9526888E9</v>
+      </c>
+      <c r="F198" s="8">
+        <v>-33.0</v>
+      </c>
+      <c r="G198" s="8">
+        <v>193.7</v>
+      </c>
+      <c r="H198" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I198" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J198" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K198" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L198" s="10" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="199" ht="15.75" customHeight="1">
-      <c r="A199" s="1"/>
+      <c r="A199" s="4">
+        <v>46221.572222222225</v>
+      </c>
+      <c r="B199" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C199" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D199" s="8">
+        <v>9.472159685E9</v>
+      </c>
+      <c r="E199" s="8">
+        <v>6.954535449E9</v>
+      </c>
+      <c r="F199" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="G199" s="8">
+        <v>193.7</v>
+      </c>
+      <c r="H199" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I199" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J199" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K199" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L199" s="10" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="200" ht="15.75" customHeight="1">
-      <c r="A200" s="1"/>
+      <c r="A200" s="4">
+        <v>46221.60833333333</v>
+      </c>
+      <c r="B200" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C200" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D200" s="8">
+        <v>9.472783437E9</v>
+      </c>
+      <c r="E200" s="8">
+        <v>6.955013125E9</v>
+      </c>
+      <c r="F200" s="8">
+        <v>-32.5</v>
+      </c>
+      <c r="G200" s="8">
+        <v>161.2</v>
+      </c>
+      <c r="H200" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I200" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J200" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K200" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L200" s="10" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="201" ht="15.75" customHeight="1">
-      <c r="A201" s="1"/>
+      <c r="A201" s="4">
+        <v>46221.77013888889</v>
+      </c>
+      <c r="B201" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C201" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D201" s="8">
+        <v>9.475230167E9</v>
+      </c>
+      <c r="E201" s="8">
+        <v>6.9526888E9</v>
+      </c>
+      <c r="F201" s="8">
+        <v>77.55</v>
+      </c>
+      <c r="G201" s="8">
+        <v>238.75</v>
+      </c>
+      <c r="H201" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I201" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J201" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K201" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L201" s="10" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="202" ht="15.75" customHeight="1">
-      <c r="A202" s="1"/>
+      <c r="A202" s="4">
+        <v>46221.95972222222</v>
+      </c>
+      <c r="B202" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C202" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D202" s="8">
+        <v>9.476408446E9</v>
+      </c>
+      <c r="E202" s="8">
+        <v>6.957622222E9</v>
+      </c>
+      <c r="F202" s="8">
+        <v>-32.5</v>
+      </c>
+      <c r="G202" s="8">
+        <v>206.25</v>
+      </c>
+      <c r="H202" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I202" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J202" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K202" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L202" s="10" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="1"/>
@@ -12026,9 +12334,9 @@
       <c r="A1000" s="11"/>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$U$194">
-    <sortState ref="A1:U194">
-      <sortCondition ref="A1:A194"/>
+  <autoFilter ref="$A$1:$U$202">
+    <sortState ref="A1:U202">
+      <sortCondition ref="A1:A202"/>
     </sortState>
   </autoFilter>
   <drawing r:id="rId1"/>
@@ -13073,34 +13381,34 @@
         <v>Player</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>26</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="L1" s="15" t="s">
         <v>6</v>
@@ -13130,7 +13438,7 @@
       </c>
       <c r="B2" s="18">
         <f>COUNTIFS('Transaction History'!L:L,A2,'Transaction History'!B:B,"Bet Stake")</f>
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C2" s="18" t="str">
         <f>COUNTIFS('Transaction History'!L:L,A2,
@@ -13187,7 +13495,7 @@
       </c>
       <c r="B3" s="18">
         <f>COUNTIFS('Transaction History'!L:L,A3,'Transaction History'!B:B,"Bet Stake")</f>
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C3" s="18" t="str">
         <f>COUNTIFS('Transaction History'!L:L,A3,
@@ -13241,7 +13549,7 @@
       </c>
       <c r="B4" s="25">
         <f>COUNTIFS('Transaction History'!L:L,A4,'Transaction History'!B:B,"Bet Stake")</f>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C4" s="25" t="str">
         <f>COUNTIFS('Transaction History'!L:L,A4,
@@ -14986,34 +15294,34 @@
         <v>#REF!</v>
       </c>
       <c r="B1" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="34" t="s">
         <v>141</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="F1" s="34" t="s">
         <v>142</v>
       </c>
-      <c r="D1" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="E1" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="F1" s="34" t="s">
-        <v>135</v>
-      </c>
       <c r="G1" s="35" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="H1" s="36" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="I1" s="37" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="J1" s="38" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="K1" s="39" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
@@ -20297,12 +20605,12 @@
     <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1">
       <c r="O28" s="72" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="O29" s="2" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1"/>
@@ -22310,37 +22618,37 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="33" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="B1" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="H1" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="J1" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="K1" s="39" t="s">
         <v>155</v>
-      </c>
-      <c r="C1" s="35" t="s">
-        <v>142</v>
-      </c>
-      <c r="D1" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="E1" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="F1" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="G1" s="35" t="s">
-        <v>144</v>
-      </c>
-      <c r="H1" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="I1" s="37" t="s">
-        <v>146</v>
-      </c>
-      <c r="J1" s="39" t="s">
-        <v>156</v>
-      </c>
-      <c r="K1" s="39" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
@@ -22348,7 +22656,7 @@
         <v>14</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C2" s="25">
         <v>0.0</v>
@@ -22403,7 +22711,7 @@
         <v>16</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C3" s="43">
         <v>0.0</v>
@@ -22458,7 +22766,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="50" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C4" s="49">
         <v>0.0</v>
@@ -22513,7 +22821,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C5" s="43">
         <v>1.0</v>
@@ -22568,7 +22876,7 @@
         <v>14</v>
       </c>
       <c r="B6" s="43" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C6" s="43">
         <v>1.0</v>
@@ -22623,7 +22931,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="49" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C7" s="49">
         <v>1.0</v>
@@ -22678,7 +22986,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C8" s="25">
         <v>2.0</v>
@@ -22733,7 +23041,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="43" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C9" s="43">
         <v>2.0</v>
@@ -22788,7 +23096,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="49" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C10" s="49">
         <v>2.0</v>
@@ -22843,7 +23151,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C11" s="25">
         <v>3.0</v>
@@ -22898,7 +23206,7 @@
         <v>16</v>
       </c>
       <c r="B12" s="43" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C12" s="43">
         <v>3.0</v>
@@ -22953,7 +23261,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C13" s="49">
         <v>3.0</v>
@@ -23008,7 +23316,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C14" s="25">
         <v>4.0</v>
@@ -23063,7 +23371,7 @@
         <v>16</v>
       </c>
       <c r="B15" s="43" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C15" s="43">
         <v>4.0</v>
@@ -23118,7 +23426,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="49" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C16" s="49">
         <v>4.0</v>
@@ -23173,7 +23481,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C17" s="25">
         <v>5.0</v>
@@ -23228,7 +23536,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="43" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C18" s="43">
         <v>5.0</v>
@@ -23283,7 +23591,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C19" s="49">
         <v>5.0</v>
@@ -23338,7 +23646,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C20" s="43">
         <v>6.0</v>
@@ -23393,7 +23701,7 @@
         <v>14</v>
       </c>
       <c r="B21" s="43" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C21" s="43">
         <v>6.0</v>
@@ -23448,7 +23756,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C22" s="49">
         <v>6.0</v>
@@ -23501,37 +23809,37 @@
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="77" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B24" s="78" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C24" s="78" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="D24" s="78" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="E24" s="78" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F24" s="78" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G24" s="78" t="s">
         <v>26</v>
       </c>
       <c r="H24" s="79" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="I24" s="80" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="J24" s="80" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="K24" s="80" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="L24" s="81" t="s">
         <v>6</v>
@@ -24557,37 +24865,37 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="H1" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="J1" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="K1" s="39" t="s">
         <v>155</v>
-      </c>
-      <c r="C1" s="35" t="s">
-        <v>142</v>
-      </c>
-      <c r="D1" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="E1" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="F1" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="G1" s="35" t="s">
-        <v>144</v>
-      </c>
-      <c r="H1" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="I1" s="37" t="s">
-        <v>146</v>
-      </c>
-      <c r="J1" s="38" t="s">
-        <v>147</v>
-      </c>
-      <c r="K1" s="39" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
@@ -24595,7 +24903,7 @@
         <v>16</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C2" s="25">
         <v>7.0</v>
@@ -24650,7 +24958,7 @@
         <v>15</v>
       </c>
       <c r="B3" s="43" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C3" s="43">
         <v>7.0</v>
@@ -24705,7 +25013,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="49" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C4" s="49">
         <v>7.0</v>
@@ -24760,7 +25068,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C5" s="25">
         <v>8.0</v>
@@ -24815,7 +25123,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="43" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C6" s="43">
         <v>8.0</v>
@@ -24870,7 +25178,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="43" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C7" s="43">
         <v>8.0</v>
@@ -24925,7 +25233,7 @@
         <v>15</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C8" s="35">
         <v>9.0</v>
@@ -24980,7 +25288,7 @@
         <v>14</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C9" s="29">
         <v>9.0</v>
@@ -25035,7 +25343,7 @@
         <v>16</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C10" s="29">
         <v>9.0</v>
@@ -25090,7 +25398,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C11" s="35">
         <v>10.0</v>
@@ -25145,7 +25453,7 @@
         <v>15</v>
       </c>
       <c r="B12" s="29" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C12" s="29">
         <v>10.0</v>
@@ -25200,7 +25508,7 @@
         <v>16</v>
       </c>
       <c r="B13" s="82" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C13" s="82">
         <v>10.0</v>
@@ -25255,7 +25563,7 @@
         <v>15</v>
       </c>
       <c r="B14" s="29" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C14" s="35">
         <v>11.0</v>
@@ -25310,7 +25618,7 @@
         <v>16</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C15" s="29">
         <v>11.0</v>
@@ -25365,7 +25673,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C16" s="29">
         <v>11.0</v>
@@ -25420,7 +25728,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C17" s="29">
         <v>12.0</v>
@@ -25475,7 +25783,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="29" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C18" s="29">
         <v>12.0</v>
@@ -25530,7 +25838,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="29" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C19" s="29">
         <v>12.0</v>
@@ -26602,37 +26910,37 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="H1" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="J1" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="K1" s="39" t="s">
         <v>155</v>
-      </c>
-      <c r="C1" s="35" t="s">
-        <v>142</v>
-      </c>
-      <c r="D1" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="E1" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="F1" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="G1" s="35" t="s">
-        <v>144</v>
-      </c>
-      <c r="H1" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="I1" s="37" t="s">
-        <v>146</v>
-      </c>
-      <c r="J1" s="38" t="s">
-        <v>147</v>
-      </c>
-      <c r="K1" s="39" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
@@ -26640,7 +26948,7 @@
         <v>14</v>
       </c>
       <c r="B2" s="35" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C2" s="35">
         <v>13.0</v>
@@ -26677,7 +26985,7 @@
         <v>16</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C3" s="29">
         <v>13.0</v>
@@ -26714,7 +27022,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="82" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C4" s="82">
         <v>13.0</v>
@@ -26751,7 +27059,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C5" s="35">
         <v>14.0</v>
@@ -26788,7 +27096,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C6" s="29">
         <v>14.0</v>
@@ -26825,7 +27133,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="82" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C7" s="82">
         <v>14.0</v>
@@ -26862,7 +27170,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C8" s="35">
         <v>15.0</v>
@@ -26899,7 +27207,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C9" s="29">
         <v>15.0</v>
@@ -26936,7 +27244,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="82" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C10" s="82">
         <v>15.0</v>
@@ -26973,7 +27281,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C11" s="35">
         <v>16.0</v>
@@ -27028,7 +27336,7 @@
         <v>16</v>
       </c>
       <c r="B12" s="29" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C12" s="29">
         <v>16.0</v>
@@ -27083,7 +27391,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="82" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C13" s="82">
         <v>16.0</v>
@@ -28160,37 +28468,37 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="H1" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="J1" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="K1" s="39" t="s">
         <v>155</v>
-      </c>
-      <c r="C1" s="35" t="s">
-        <v>142</v>
-      </c>
-      <c r="D1" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="E1" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="F1" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="G1" s="35" t="s">
-        <v>144</v>
-      </c>
-      <c r="H1" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="I1" s="37" t="s">
-        <v>146</v>
-      </c>
-      <c r="J1" s="38" t="s">
-        <v>147</v>
-      </c>
-      <c r="K1" s="39" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1"/>

</xml_diff>